<commit_message>
Actualizacion semanal de vigilancia
</commit_message>
<xml_diff>
--- a/Animal desconocido 2026/ANIMAL DESCONOCIDO.xlsx
+++ b/Animal desconocido 2026/ANIMAL DESCONOCIDO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\2026\app VACUNACION ANTIRRAVICA 2025 - 2026\Animal desconocido 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BFCFD78-A87D-49A7-93AA-23B6DD28BE15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9328F683-4C68-4245-AE53-482AE89509DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="73">
   <si>
     <t>FUNCIONARIO</t>
   </si>
@@ -190,15 +190,69 @@
   </si>
   <si>
     <t>0.688598, -76.604928</t>
+  </si>
+  <si>
+    <t>573eedd4</t>
+  </si>
+  <si>
+    <t>ORITO</t>
+  </si>
+  <si>
+    <t>LOS ALMENDROS</t>
+  </si>
+  <si>
+    <t>Perro en buen estado</t>
+  </si>
+  <si>
+    <t>Bicolor</t>
+  </si>
+  <si>
+    <t>ANIMAL_CALLE_Images/573eedd4.FOTO_ANIMAL.142531.jpg</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>MARIA ARELIZ ORTIZ</t>
+  </si>
+  <si>
+    <t>0.675338, -76.865854</t>
+  </si>
+  <si>
+    <t>75440388</t>
+  </si>
+  <si>
+    <t>SIBUNDOY</t>
+  </si>
+  <si>
+    <t>TAMABIOY</t>
+  </si>
+  <si>
+    <t>Tamabioy</t>
+  </si>
+  <si>
+    <t>Tamaño medio,semi churozo</t>
+  </si>
+  <si>
+    <t>Amarillo</t>
+  </si>
+  <si>
+    <t>ANIMAL_CALLE_Images/75440388.FOTO_ANIMAL.172338.jpg</t>
+  </si>
+  <si>
+    <t>No reportada en hospital, se llama Lucy, agrede a la comunidad</t>
+  </si>
+  <si>
+    <t>Es abandonada, vive cerca de una casa de madera. Sandra jacamamejoy.</t>
+  </si>
+  <si>
+    <t>1.180420, -76.888493</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm;@"/>
-  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -274,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -291,13 +345,16 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -518,16 +575,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" style="9" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="28.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.7109375" style="2" bestFit="1" customWidth="1"/>
@@ -537,12 +594,12 @@
     <col min="14" max="14" width="19.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="55" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="55.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="24" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="54.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="57.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="26.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="63.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="65.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="20.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="24" max="16384" width="14.42578125" style="2"/>
   </cols>
@@ -551,7 +608,7 @@
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -622,13 +679,13 @@
       <c r="A2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="9">
         <v>46247</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>33</v>
       </c>
       <c r="E2" s="5"/>
@@ -688,13 +745,13 @@
       <c r="A3" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="9">
         <v>46248</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>44</v>
       </c>
       <c r="E3" s="5"/>
@@ -739,11 +796,130 @@
       <c r="V3" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="W3" s="8" t="s">
+      <c r="W3" s="7" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="9">
+        <v>46254</v>
+      </c>
+      <c r="C4" s="2">
+        <v>34</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="9">
+        <v>46256</v>
+      </c>
+      <c r="C5" s="2">
+        <v>34</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="U5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizacion de datos de nueva carpeta
</commit_message>
<xml_diff>
--- a/Animal desconocido 2026/ANIMAL DESCONOCIDO.xlsx
+++ b/Animal desconocido 2026/ANIMAL DESCONOCIDO.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\2026\app VACUNACION ANTIRRAVICA 2025 - 2026\Animal desconocido 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9328F683-4C68-4245-AE53-482AE89509DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB7B6B4D-737E-479E-B4E9-B30D8D569758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ANIMAL_CALLE" sheetId="23" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="81">
   <si>
     <t>FUNCIONARIO</t>
   </si>
@@ -247,12 +247,39 @@
   </si>
   <si>
     <t>1.180420, -76.888493</t>
+  </si>
+  <si>
+    <t>d7c53e75</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>VEGAS FATIMA</t>
+  </si>
+  <si>
+    <t>Delgado, cola larga pelo corto</t>
+  </si>
+  <si>
+    <t>Colorado</t>
+  </si>
+  <si>
+    <t>ANIMAL_CALLE_Images/d7c53e75.FOTO_ANIMAL.190637.jpg</t>
+  </si>
+  <si>
+    <t>Perro se encuentra bajando el montallatas por la calle despavimentada.  Le gusta perseguir motos y carros</t>
+  </si>
+  <si>
+    <t>1.196991, -76.909065</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm;@"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -328,7 +355,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -355,6 +382,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -575,7 +605,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" style="2" customWidth="1"/>
@@ -918,6 +948,65 @@
         <v>72</v>
       </c>
     </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="10">
+        <v>46268</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="T6" s="5"/>
+      <c r="U6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="0" r:id="rId1"/>

</xml_diff>